<commit_message>
feat: fill district_area_seed for all 22 Taiwan regions
Add comprehensive district and commercial area reference data to all Excel files:
- 台北市 12區 48商圈
- 新北市 15區 60商圈
- 桃園市 13區 52商圈
- 台中市 28區 112商圈
- 台南市 16區 64商圈
- 高雄市 16區 64商圈
- 基隆市 7區 28商圈
- 新竹市 3區 12商圈
- 新竹縣 13鄉鎮 52商圈
- 苗栗縣 18鄉鎮 72商圈
- 彰化縣 26鄉鎮 104商圈
- 南投縣 13鄉鎮 52商圈
- 雲林縣 20鄉鎮 80商圈
- 嘉義市 2區 8商圈
- 嘉義縣 18鄉鎮 72商圈
- 屏東縣 16鄉鎮 64商圈
- 宜蘭縣 12鄉鎮 48商圈
- 花蓮縣 13鄉鎮 52商圈
- 台東縣 16鄉鎮 64商圈
- 澎湖縣 6鄉鎮 24商圈
- 金門縣 6鄉鎮 24商圈
- 連江縣 4鄉 16商圈

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/excel/01-taipei.xlsx
+++ b/data/excel/01-taipei.xlsx
@@ -872,7 +872,6 @@
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1273,8 +1272,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -1297,6 +1302,870 @@
           <t>note</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>中正區</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>台北車站周邊</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>中正區</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>公館商圈</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>中正區</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>師大商圈</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>中正區</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>南門市場</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>大同區</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>迪化街</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>大同區</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>寧夏夜市</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>大同區</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>大橋頭</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>大同區</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>承德路</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>中山區</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>中山商圈</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>中山區</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>林森北路</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>中山區</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>南京商圈</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>中山區</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>晴光商圈</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>松山區</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>饒河夜市</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>松山區</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>南京東路</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>松山區</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>八德路</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>松山區</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>台北小巨蛋</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>忠孝東路</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>永康街</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>師大夜市</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>大安區</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>信義路</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>萬華區</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>西門町</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>萬華區</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>龍山寺</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>萬華區</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>華西街</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>萬華區</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>艋舺商圈</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>信義區</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>信義商圈</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>信義區</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>台北101周邊</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>信義區</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>松菸文創</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>信義區</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>四四南村</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>士林區</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>士林夜市</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>士林區</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>天母商圈</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>士林區</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>文昌路</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>士林區</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>劍潭</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>北投區</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>新北投溫泉</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>北投區</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>北投市場</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>北投區</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>石牌商圈</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>北投區</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>光明路</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>內湖區</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>內湖科學園區</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>內湖區</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>成功路</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>內湖區</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>西湖市場</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>內湖區</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>瑞光路</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>南港區</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>南港展覽館</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>南港區</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>南港軟體園區</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>南港區</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>忠孝東路</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>南港區</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>昆陽</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>文山區</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>景美夜市</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>文山區</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>景美商圈</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>文山區</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>木柵動物園</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>文山區</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>萬隆商圈</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>商圈</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>